<commit_message>
Complete documentation overhaul with architecture, dashboards and README updates
</commit_message>
<xml_diff>
--- a/data/raw/excel/Superette_Data.xlsx
+++ b/data/raw/excel/Superette_Data.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Girand-20260315\2_Privat\7_projet_Boutique\superette\data\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\Girand-20260315\2_Privat\7_projet_Boutique\superette\data\raw\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B541C3E-94A5-468A-A85E-46BC23E74CAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF082C5C-0DAA-4252-B8DB-EE104B2B051B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="15" xr2:uid="{6E9F0846-86AC-4AA2-B626-2CA9074A1B28}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{6E9F0846-86AC-4AA2-B626-2CA9074A1B28}"/>
   </bookViews>
   <sheets>
     <sheet name="tous Tabelles" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">dim_lignes_vente!$I$1:$I$183</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -56,6 +55,40 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>User</author>
+  </authors>
+  <commentList>
+    <comment ref="C59" authorId="0" shapeId="0" xr:uid="{5347D85F-486E-4B84-A3E8-B4D7E6106AF4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t>User:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+80000dette</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1396,7 +1429,7 @@
     <numFmt numFmtId="165" formatCode="_-* #,##0\ [$FCFA-2C0C]_-;\-* #,##0\ [$FCFA-2C0C]_-;_-* &quot;-&quot;??\ [$FCFA-2C0C]_-;_-@_-"/>
     <numFmt numFmtId="166" formatCode="_-* #,##0.0\ [$FCFA-2C0C]_-;\-* #,##0.0\ [$FCFA-2C0C]_-;_-* &quot;-&quot;??\ [$FCFA-2C0C]_-;_-@_-"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1484,6 +1517,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="18">
@@ -2032,8 +2078,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{03C348FD-B8B3-4E22-87A0-123710BCF5FA}" name="Tabelle1" displayName="Tabelle1" ref="A3:G58" totalsRowShown="0" dataDxfId="8">
-  <autoFilter ref="A3:G58" xr:uid="{03C348FD-B8B3-4E22-87A0-123710BCF5FA}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{03C348FD-B8B3-4E22-87A0-123710BCF5FA}" name="Tabelle1" displayName="Tabelle1" ref="A3:G64" totalsRowShown="0" dataDxfId="8">
+  <autoFilter ref="A3:G64" xr:uid="{03C348FD-B8B3-4E22-87A0-123710BCF5FA}"/>
   <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{CFE74404-5491-4C73-8750-8662CD163BAE}" name="Date" dataDxfId="7"/>
     <tableColumn id="2" xr3:uid="{ABCA7BB5-E954-47D9-AB43-61D3DDF02A58}" name="Depart" dataDxfId="6"/>
@@ -16911,7 +16957,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF80F024-65A6-40B4-B8E0-B97D989DD769}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CF80F024-65A6-40B4-B8E0-B97D989DD769}">
   <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <cols>
@@ -16935,11 +16981,11 @@
     <row r="2" spans="1:8" ht="15.6">
       <c r="C2" s="16">
         <f>SUM(Tabelle1[Entre])</f>
-        <v>1876825</v>
+        <v>2278575</v>
       </c>
       <c r="D2" s="16">
         <f>SUM(Tabelle1[Achat])</f>
-        <v>1518150</v>
+        <v>1906450</v>
       </c>
       <c r="E2" s="16">
         <f>SUM(Tabelle1[autre depence])</f>
@@ -16947,7 +16993,7 @@
       </c>
       <c r="G2" s="17">
         <f>C2-D2-E2+B4</f>
-        <v>515575</v>
+        <v>529025</v>
       </c>
     </row>
     <row r="3" spans="1:8">
@@ -17720,7 +17766,8 @@
       </c>
       <c r="B52" s="6"/>
       <c r="C52" s="5">
-        <v>21900</v>
+        <f>21900+13500</f>
+        <v>35400</v>
       </c>
       <c r="D52" s="5">
         <v>29400</v>
@@ -17731,9 +17778,13 @@
       <c r="H52" s="6"/>
     </row>
     <row r="53" spans="1:8">
-      <c r="A53" s="4"/>
+      <c r="A53" s="4">
+        <v>47320</v>
+      </c>
       <c r="B53" s="6"/>
-      <c r="C53" s="5"/>
+      <c r="C53" s="5">
+        <v>50800</v>
+      </c>
       <c r="D53" s="5"/>
       <c r="E53" s="5"/>
       <c r="F53" s="6"/>
@@ -17741,9 +17792,13 @@
       <c r="H53" s="6"/>
     </row>
     <row r="54" spans="1:8">
-      <c r="A54" s="4"/>
+      <c r="A54" s="4">
+        <v>46225</v>
+      </c>
       <c r="B54" s="6"/>
-      <c r="C54" s="5"/>
+      <c r="C54" s="5">
+        <v>51825</v>
+      </c>
       <c r="D54" s="5"/>
       <c r="E54" s="5"/>
       <c r="F54" s="6"/>
@@ -17751,9 +17806,13 @@
       <c r="H54" s="6"/>
     </row>
     <row r="55" spans="1:8">
-      <c r="A55" s="4"/>
+      <c r="A55" s="4">
+        <v>46226</v>
+      </c>
       <c r="B55" s="6"/>
-      <c r="C55" s="5"/>
+      <c r="C55" s="5">
+        <v>44225</v>
+      </c>
       <c r="D55" s="5"/>
       <c r="E55" s="5"/>
       <c r="F55" s="6"/>
@@ -17761,19 +17820,29 @@
       <c r="H55" s="6"/>
     </row>
     <row r="56" spans="1:8">
-      <c r="A56" s="4"/>
+      <c r="A56" s="4">
+        <v>46227</v>
+      </c>
       <c r="B56" s="6"/>
-      <c r="C56" s="5"/>
-      <c r="D56" s="5"/>
+      <c r="C56" s="5">
+        <v>24725</v>
+      </c>
+      <c r="D56" s="5">
+        <v>72600</v>
+      </c>
       <c r="E56" s="5"/>
       <c r="F56" s="6"/>
       <c r="G56" s="6"/>
       <c r="H56" s="6"/>
     </row>
     <row r="57" spans="1:8">
-      <c r="A57" s="4"/>
+      <c r="A57" s="4">
+        <v>46228</v>
+      </c>
       <c r="B57" s="6"/>
-      <c r="C57" s="5"/>
+      <c r="C57" s="5">
+        <v>58775</v>
+      </c>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
       <c r="F57" s="6"/>
@@ -17781,9 +17850,13 @@
       <c r="H57" s="6"/>
     </row>
     <row r="58" spans="1:8">
-      <c r="A58" s="4"/>
+      <c r="A58" s="4">
+        <v>46229</v>
+      </c>
       <c r="B58" s="6"/>
-      <c r="C58" s="5"/>
+      <c r="C58" s="5">
+        <v>41175</v>
+      </c>
       <c r="D58" s="5"/>
       <c r="E58" s="5"/>
       <c r="F58" s="6"/>
@@ -17791,10 +17864,17 @@
       <c r="H58" s="6"/>
     </row>
     <row r="59" spans="1:8">
-      <c r="A59" s="4"/>
+      <c r="A59" s="4">
+        <v>46231</v>
+      </c>
       <c r="B59" s="6"/>
-      <c r="C59" s="5"/>
-      <c r="D59" s="5"/>
+      <c r="C59" s="5">
+        <f>80000+36725</f>
+        <v>116725</v>
+      </c>
+      <c r="D59" s="5">
+        <v>315700</v>
+      </c>
       <c r="E59" s="5"/>
       <c r="F59" s="6"/>
       <c r="G59" s="6"/>
@@ -17985,8 +18065,9 @@
     <mergeCell ref="C1:E1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>